<commit_message>
feat(form63): implement final form 63 export with template, ui and backend logic
</commit_message>
<xml_diff>
--- a/backend/generated/form63/form63_template_1.xlsx
+++ b/backend/generated/form63/form63_template_1.xlsx
@@ -1402,128 +1402,412 @@
       <c r="U15" s="87" t="n"/>
     </row>
     <row r="16" ht="15.6" customHeight="1">
-      <c r="C16" s="88" t="n"/>
-      <c r="D16" s="21" t="n"/>
-      <c r="G16" s="21" t="n"/>
-      <c r="J16" s="14" t="n"/>
-      <c r="K16" s="21" t="n"/>
-      <c r="L16" s="21" t="n"/>
-      <c r="M16" s="16" t="n"/>
-      <c r="N16" s="16" t="n"/>
-      <c r="O16" s="16" t="n"/>
-      <c r="P16" s="16" t="n"/>
-      <c r="Q16" s="16" t="n"/>
-      <c r="R16" s="16" t="n"/>
-      <c r="S16" s="16" t="n"/>
-      <c r="T16" s="21" t="n"/>
-      <c r="U16" s="16" t="n"/>
+      <c r="C16" s="88" t="n">
+        <v>1</v>
+      </c>
+      <c r="D16" s="21" t="inlineStr">
+        <is>
+          <t>Алтайбек Айжан Алтайбекқызы</t>
+        </is>
+      </c>
+      <c r="G16" s="21" t="inlineStr">
+        <is>
+          <t>ассоциированный профессор</t>
+        </is>
+      </c>
+      <c r="J16" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="K16" s="21" t="n">
+        <v>125</v>
+      </c>
+      <c r="L16" s="21" t="n">
+        <v>50</v>
+      </c>
+      <c r="M16" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="N16" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="O16" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="P16" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q16" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="R16" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="S16" s="16" t="n">
+        <v>175</v>
+      </c>
+      <c r="T16" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="U16" s="16" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="17" ht="15.6" customHeight="1">
-      <c r="J17" s="14" t="n"/>
-      <c r="K17" s="21" t="n"/>
-      <c r="L17" s="21" t="n"/>
-      <c r="M17" s="16" t="n"/>
-      <c r="N17" s="16" t="n"/>
-      <c r="O17" s="16" t="n"/>
-      <c r="P17" s="16" t="n"/>
-      <c r="Q17" s="16" t="n"/>
-      <c r="R17" s="16" t="n"/>
-      <c r="S17" s="16" t="n"/>
-      <c r="T17" s="21" t="n"/>
-      <c r="U17" s="16" t="n"/>
+      <c r="C17" t="n">
+        <v>1</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Алтайбек Айжан Алтайбекқызы</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>ассоциированный профессор</t>
+        </is>
+      </c>
+      <c r="J17" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="K17" s="21" t="n">
+        <v>102</v>
+      </c>
+      <c r="L17" s="21" t="n">
+        <v>50</v>
+      </c>
+      <c r="M17" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="N17" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="O17" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="P17" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q17" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="R17" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="S17" s="16" t="n">
+        <v>152</v>
+      </c>
+      <c r="T17" s="21" t="n">
+        <v>81</v>
+      </c>
+      <c r="U17" s="16" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="18" ht="15.6" customHeight="1">
-      <c r="C18" s="88" t="n"/>
-      <c r="D18" s="21" t="n"/>
-      <c r="G18" s="21" t="n"/>
-      <c r="J18" s="14" t="n"/>
-      <c r="K18" s="21" t="n"/>
-      <c r="L18" s="21" t="n"/>
-      <c r="M18" s="16" t="n"/>
-      <c r="N18" s="16" t="n"/>
-      <c r="O18" s="16" t="n"/>
-      <c r="P18" s="16" t="n"/>
-      <c r="Q18" s="16" t="n"/>
-      <c r="R18" s="16" t="n"/>
-      <c r="S18" s="16" t="n"/>
-      <c r="T18" s="21" t="n"/>
-      <c r="U18" s="16" t="n"/>
+      <c r="C18" s="88" t="n">
+        <v>2</v>
+      </c>
+      <c r="D18" s="21" t="inlineStr">
+        <is>
+          <t>Нұртас Марат</t>
+        </is>
+      </c>
+      <c r="G18" s="21" t="inlineStr">
+        <is>
+          <t>ассоциированный профессор</t>
+        </is>
+      </c>
+      <c r="J18" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="K18" s="21" t="n">
+        <v>142</v>
+      </c>
+      <c r="L18" s="21" t="n">
+        <v>125</v>
+      </c>
+      <c r="M18" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="N18" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="O18" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="P18" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q18" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="R18" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="S18" s="16" t="n">
+        <v>267</v>
+      </c>
+      <c r="T18" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="U18" s="16" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="19" ht="15.6" customHeight="1">
-      <c r="J19" s="14" t="n"/>
-      <c r="K19" s="21" t="n"/>
-      <c r="L19" s="21" t="n"/>
-      <c r="M19" s="16" t="n"/>
-      <c r="N19" s="16" t="n"/>
-      <c r="O19" s="16" t="n"/>
-      <c r="P19" s="16" t="n"/>
-      <c r="Q19" s="16" t="n"/>
-      <c r="R19" s="16" t="n"/>
-      <c r="S19" s="16" t="n"/>
-      <c r="T19" s="21" t="n"/>
-      <c r="U19" s="16" t="n"/>
+      <c r="C19" t="n">
+        <v>2</v>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Нұртас Марат</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>ассоциированный профессор</t>
+        </is>
+      </c>
+      <c r="J19" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="K19" s="21" t="n">
+        <v>96</v>
+      </c>
+      <c r="L19" s="21" t="n">
+        <v>125</v>
+      </c>
+      <c r="M19" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="N19" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="O19" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="P19" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q19" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="R19" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="S19" s="16" t="n">
+        <v>221</v>
+      </c>
+      <c r="T19" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="U19" s="16" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20" ht="15.6" customHeight="1">
-      <c r="C20" s="88" t="n"/>
-      <c r="D20" s="21" t="n"/>
-      <c r="G20" s="21" t="n"/>
-      <c r="J20" s="14" t="n"/>
-      <c r="K20" s="21" t="n"/>
-      <c r="L20" s="21" t="n"/>
-      <c r="M20" s="16" t="n"/>
-      <c r="N20" s="16" t="n"/>
-      <c r="O20" s="16" t="n"/>
-      <c r="P20" s="16" t="n"/>
-      <c r="Q20" s="16" t="n"/>
-      <c r="R20" s="16" t="n"/>
-      <c r="S20" s="16" t="n"/>
-      <c r="T20" s="21" t="n"/>
-      <c r="U20" s="16" t="n"/>
+      <c r="C20" s="88" t="n">
+        <v>3</v>
+      </c>
+      <c r="D20" s="21" t="inlineStr">
+        <is>
+          <t>Сраж Айнур</t>
+        </is>
+      </c>
+      <c r="G20" s="21" t="inlineStr">
+        <is>
+          <t>сениор лектор</t>
+        </is>
+      </c>
+      <c r="J20" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="K20" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="L20" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="M20" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="N20" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="O20" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="P20" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q20" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="R20" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="S20" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="T20" s="21" t="n">
+        <v>87</v>
+      </c>
+      <c r="U20" s="16" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="21" ht="15.6" customHeight="1">
-      <c r="J21" s="14" t="n"/>
-      <c r="K21" s="21" t="n"/>
-      <c r="L21" s="21" t="n"/>
-      <c r="M21" s="16" t="n"/>
-      <c r="N21" s="16" t="n"/>
-      <c r="O21" s="16" t="n"/>
-      <c r="P21" s="16" t="n"/>
-      <c r="Q21" s="16" t="n"/>
-      <c r="R21" s="16" t="n"/>
-      <c r="S21" s="16" t="n"/>
-      <c r="T21" s="21" t="n"/>
-      <c r="U21" s="16" t="n"/>
+      <c r="C21" t="n">
+        <v>3</v>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Сраж Айнур</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>сениор лектор</t>
+        </is>
+      </c>
+      <c r="J21" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="K21" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="L21" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="M21" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="N21" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="O21" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="P21" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q21" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="R21" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="S21" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="T21" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="U21" s="16" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="22" ht="15.6" customHeight="1">
-      <c r="C22" s="88" t="n"/>
-      <c r="D22" s="21" t="n"/>
-      <c r="G22" s="21" t="n"/>
-      <c r="J22" s="14" t="n"/>
-      <c r="K22" s="21" t="n"/>
-      <c r="L22" s="21" t="n"/>
-      <c r="M22" s="16" t="n"/>
-      <c r="N22" s="16" t="n"/>
-      <c r="O22" s="16" t="n"/>
-      <c r="P22" s="16" t="n"/>
-      <c r="Q22" s="16" t="n"/>
-      <c r="R22" s="16" t="n"/>
-      <c r="S22" s="16" t="n"/>
-      <c r="T22" s="21" t="n"/>
-      <c r="U22" s="16" t="n"/>
+      <c r="C22" s="88" t="n">
+        <v>4</v>
+      </c>
+      <c r="D22" s="21" t="inlineStr">
+        <is>
+          <t>Ыдырыс Жәнібек Жұмабайұлы</t>
+        </is>
+      </c>
+      <c r="G22" s="21" t="inlineStr">
+        <is>
+          <t>сениор лектор</t>
+        </is>
+      </c>
+      <c r="J22" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="K22" s="21" t="n">
+        <v>688</v>
+      </c>
+      <c r="L22" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="M22" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="N22" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="O22" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="P22" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q22" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="R22" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="S22" s="16" t="n">
+        <v>688</v>
+      </c>
+      <c r="T22" s="21" t="n">
+        <v>40</v>
+      </c>
+      <c r="U22" s="16" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23" ht="15.6" customHeight="1">
-      <c r="J23" s="14" t="n"/>
-      <c r="K23" s="21" t="n"/>
-      <c r="L23" s="21" t="n"/>
-      <c r="M23" s="16" t="n"/>
-      <c r="N23" s="16" t="n"/>
-      <c r="O23" s="16" t="n"/>
-      <c r="P23" s="16" t="n"/>
-      <c r="Q23" s="16" t="n"/>
-      <c r="R23" s="16" t="n"/>
-      <c r="S23" s="16" t="n"/>
-      <c r="T23" s="21" t="n"/>
-      <c r="U23" s="16" t="n"/>
+      <c r="C23" t="n">
+        <v>4</v>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Ыдырыс Жәнібек Жұмабайұлы</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>сениор лектор</t>
+        </is>
+      </c>
+      <c r="J23" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="K23" s="21" t="n">
+        <v>417.5</v>
+      </c>
+      <c r="L23" s="21" t="n">
+        <v>30</v>
+      </c>
+      <c r="M23" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="N23" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="O23" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="P23" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q23" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="R23" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="S23" s="16" t="n">
+        <v>447.5</v>
+      </c>
+      <c r="T23" s="21" t="n">
+        <v>37</v>
+      </c>
+      <c r="U23" s="16" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="24" ht="15.6" customHeight="1">
       <c r="C24" s="88" t="n"/>

</xml_diff>

<commit_message>
feat(form63): implement final form 63 export with template and ui
Adds Form63Page.jsx, wiring the upload-and-export flow from the previous
commit into the frontend and navbar.
</commit_message>
<xml_diff>
--- a/backend/generated/form63/form63_template_1.xlsx
+++ b/backend/generated/form63/form63_template_1.xlsx
@@ -1402,128 +1402,412 @@
       <c r="U15" s="87" t="n"/>
     </row>
     <row r="16" ht="15.6" customHeight="1">
-      <c r="C16" s="88" t="n"/>
-      <c r="D16" s="21" t="n"/>
-      <c r="G16" s="21" t="n"/>
-      <c r="J16" s="14" t="n"/>
-      <c r="K16" s="21" t="n"/>
-      <c r="L16" s="21" t="n"/>
-      <c r="M16" s="16" t="n"/>
-      <c r="N16" s="16" t="n"/>
-      <c r="O16" s="16" t="n"/>
-      <c r="P16" s="16" t="n"/>
-      <c r="Q16" s="16" t="n"/>
-      <c r="R16" s="16" t="n"/>
-      <c r="S16" s="16" t="n"/>
-      <c r="T16" s="21" t="n"/>
-      <c r="U16" s="16" t="n"/>
+      <c r="C16" s="88" t="n">
+        <v>1</v>
+      </c>
+      <c r="D16" s="21" t="inlineStr">
+        <is>
+          <t>Алтайбек Айжан Алтайбекқызы</t>
+        </is>
+      </c>
+      <c r="G16" s="21" t="inlineStr">
+        <is>
+          <t>ассоциированный профессор</t>
+        </is>
+      </c>
+      <c r="J16" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="K16" s="21" t="n">
+        <v>125</v>
+      </c>
+      <c r="L16" s="21" t="n">
+        <v>50</v>
+      </c>
+      <c r="M16" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="N16" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="O16" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="P16" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q16" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="R16" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="S16" s="16" t="n">
+        <v>175</v>
+      </c>
+      <c r="T16" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="U16" s="16" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="17" ht="15.6" customHeight="1">
-      <c r="J17" s="14" t="n"/>
-      <c r="K17" s="21" t="n"/>
-      <c r="L17" s="21" t="n"/>
-      <c r="M17" s="16" t="n"/>
-      <c r="N17" s="16" t="n"/>
-      <c r="O17" s="16" t="n"/>
-      <c r="P17" s="16" t="n"/>
-      <c r="Q17" s="16" t="n"/>
-      <c r="R17" s="16" t="n"/>
-      <c r="S17" s="16" t="n"/>
-      <c r="T17" s="21" t="n"/>
-      <c r="U17" s="16" t="n"/>
+      <c r="C17" t="n">
+        <v>1</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Алтайбек Айжан Алтайбекқызы</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>ассоциированный профессор</t>
+        </is>
+      </c>
+      <c r="J17" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="K17" s="21" t="n">
+        <v>102</v>
+      </c>
+      <c r="L17" s="21" t="n">
+        <v>50</v>
+      </c>
+      <c r="M17" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="N17" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="O17" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="P17" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q17" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="R17" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="S17" s="16" t="n">
+        <v>152</v>
+      </c>
+      <c r="T17" s="21" t="n">
+        <v>81</v>
+      </c>
+      <c r="U17" s="16" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="18" ht="15.6" customHeight="1">
-      <c r="C18" s="88" t="n"/>
-      <c r="D18" s="21" t="n"/>
-      <c r="G18" s="21" t="n"/>
-      <c r="J18" s="14" t="n"/>
-      <c r="K18" s="21" t="n"/>
-      <c r="L18" s="21" t="n"/>
-      <c r="M18" s="16" t="n"/>
-      <c r="N18" s="16" t="n"/>
-      <c r="O18" s="16" t="n"/>
-      <c r="P18" s="16" t="n"/>
-      <c r="Q18" s="16" t="n"/>
-      <c r="R18" s="16" t="n"/>
-      <c r="S18" s="16" t="n"/>
-      <c r="T18" s="21" t="n"/>
-      <c r="U18" s="16" t="n"/>
+      <c r="C18" s="88" t="n">
+        <v>2</v>
+      </c>
+      <c r="D18" s="21" t="inlineStr">
+        <is>
+          <t>Нұртас Марат</t>
+        </is>
+      </c>
+      <c r="G18" s="21" t="inlineStr">
+        <is>
+          <t>ассоциированный профессор</t>
+        </is>
+      </c>
+      <c r="J18" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="K18" s="21" t="n">
+        <v>142</v>
+      </c>
+      <c r="L18" s="21" t="n">
+        <v>125</v>
+      </c>
+      <c r="M18" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="N18" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="O18" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="P18" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q18" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="R18" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="S18" s="16" t="n">
+        <v>267</v>
+      </c>
+      <c r="T18" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="U18" s="16" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="19" ht="15.6" customHeight="1">
-      <c r="J19" s="14" t="n"/>
-      <c r="K19" s="21" t="n"/>
-      <c r="L19" s="21" t="n"/>
-      <c r="M19" s="16" t="n"/>
-      <c r="N19" s="16" t="n"/>
-      <c r="O19" s="16" t="n"/>
-      <c r="P19" s="16" t="n"/>
-      <c r="Q19" s="16" t="n"/>
-      <c r="R19" s="16" t="n"/>
-      <c r="S19" s="16" t="n"/>
-      <c r="T19" s="21" t="n"/>
-      <c r="U19" s="16" t="n"/>
+      <c r="C19" t="n">
+        <v>2</v>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Нұртас Марат</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>ассоциированный профессор</t>
+        </is>
+      </c>
+      <c r="J19" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="K19" s="21" t="n">
+        <v>96</v>
+      </c>
+      <c r="L19" s="21" t="n">
+        <v>125</v>
+      </c>
+      <c r="M19" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="N19" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="O19" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="P19" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q19" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="R19" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="S19" s="16" t="n">
+        <v>221</v>
+      </c>
+      <c r="T19" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="U19" s="16" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20" ht="15.6" customHeight="1">
-      <c r="C20" s="88" t="n"/>
-      <c r="D20" s="21" t="n"/>
-      <c r="G20" s="21" t="n"/>
-      <c r="J20" s="14" t="n"/>
-      <c r="K20" s="21" t="n"/>
-      <c r="L20" s="21" t="n"/>
-      <c r="M20" s="16" t="n"/>
-      <c r="N20" s="16" t="n"/>
-      <c r="O20" s="16" t="n"/>
-      <c r="P20" s="16" t="n"/>
-      <c r="Q20" s="16" t="n"/>
-      <c r="R20" s="16" t="n"/>
-      <c r="S20" s="16" t="n"/>
-      <c r="T20" s="21" t="n"/>
-      <c r="U20" s="16" t="n"/>
+      <c r="C20" s="88" t="n">
+        <v>3</v>
+      </c>
+      <c r="D20" s="21" t="inlineStr">
+        <is>
+          <t>Сраж Айнур</t>
+        </is>
+      </c>
+      <c r="G20" s="21" t="inlineStr">
+        <is>
+          <t>сениор лектор</t>
+        </is>
+      </c>
+      <c r="J20" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="K20" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="L20" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="M20" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="N20" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="O20" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="P20" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q20" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="R20" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="S20" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="T20" s="21" t="n">
+        <v>87</v>
+      </c>
+      <c r="U20" s="16" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="21" ht="15.6" customHeight="1">
-      <c r="J21" s="14" t="n"/>
-      <c r="K21" s="21" t="n"/>
-      <c r="L21" s="21" t="n"/>
-      <c r="M21" s="16" t="n"/>
-      <c r="N21" s="16" t="n"/>
-      <c r="O21" s="16" t="n"/>
-      <c r="P21" s="16" t="n"/>
-      <c r="Q21" s="16" t="n"/>
-      <c r="R21" s="16" t="n"/>
-      <c r="S21" s="16" t="n"/>
-      <c r="T21" s="21" t="n"/>
-      <c r="U21" s="16" t="n"/>
+      <c r="C21" t="n">
+        <v>3</v>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Сраж Айнур</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>сениор лектор</t>
+        </is>
+      </c>
+      <c r="J21" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="K21" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="L21" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="M21" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="N21" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="O21" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="P21" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q21" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="R21" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="S21" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="T21" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="U21" s="16" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="22" ht="15.6" customHeight="1">
-      <c r="C22" s="88" t="n"/>
-      <c r="D22" s="21" t="n"/>
-      <c r="G22" s="21" t="n"/>
-      <c r="J22" s="14" t="n"/>
-      <c r="K22" s="21" t="n"/>
-      <c r="L22" s="21" t="n"/>
-      <c r="M22" s="16" t="n"/>
-      <c r="N22" s="16" t="n"/>
-      <c r="O22" s="16" t="n"/>
-      <c r="P22" s="16" t="n"/>
-      <c r="Q22" s="16" t="n"/>
-      <c r="R22" s="16" t="n"/>
-      <c r="S22" s="16" t="n"/>
-      <c r="T22" s="21" t="n"/>
-      <c r="U22" s="16" t="n"/>
+      <c r="C22" s="88" t="n">
+        <v>4</v>
+      </c>
+      <c r="D22" s="21" t="inlineStr">
+        <is>
+          <t>Ыдырыс Жәнібек Жұмабайұлы</t>
+        </is>
+      </c>
+      <c r="G22" s="21" t="inlineStr">
+        <is>
+          <t>сениор лектор</t>
+        </is>
+      </c>
+      <c r="J22" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="K22" s="21" t="n">
+        <v>688</v>
+      </c>
+      <c r="L22" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="M22" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="N22" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="O22" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="P22" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q22" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="R22" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="S22" s="16" t="n">
+        <v>688</v>
+      </c>
+      <c r="T22" s="21" t="n">
+        <v>40</v>
+      </c>
+      <c r="U22" s="16" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23" ht="15.6" customHeight="1">
-      <c r="J23" s="14" t="n"/>
-      <c r="K23" s="21" t="n"/>
-      <c r="L23" s="21" t="n"/>
-      <c r="M23" s="16" t="n"/>
-      <c r="N23" s="16" t="n"/>
-      <c r="O23" s="16" t="n"/>
-      <c r="P23" s="16" t="n"/>
-      <c r="Q23" s="16" t="n"/>
-      <c r="R23" s="16" t="n"/>
-      <c r="S23" s="16" t="n"/>
-      <c r="T23" s="21" t="n"/>
-      <c r="U23" s="16" t="n"/>
+      <c r="C23" t="n">
+        <v>4</v>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Ыдырыс Жәнібек Жұмабайұлы</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>сениор лектор</t>
+        </is>
+      </c>
+      <c r="J23" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="K23" s="21" t="n">
+        <v>417.5</v>
+      </c>
+      <c r="L23" s="21" t="n">
+        <v>30</v>
+      </c>
+      <c r="M23" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="N23" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="O23" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="P23" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q23" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="R23" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="S23" s="16" t="n">
+        <v>447.5</v>
+      </c>
+      <c r="T23" s="21" t="n">
+        <v>37</v>
+      </c>
+      <c r="U23" s="16" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="24" ht="15.6" customHeight="1">
       <c r="C24" s="88" t="n"/>

</xml_diff>